<commit_message>
feat(sync): implement pessimistic cloud‑locking and multi‑user DB sync via Google Drive (#66)
- Add GoogleDriveLockService for single‑active‑session enforcement with heartbeat
- Add DatabaseSyncService for version comparison and sync on startup/shutdown
- Implement crash recovery with stale lock detection and conflict resolution
- Add local backup before conflict resolution to prevent data loss
- Reuse splash screen for shutdown progress and exit confirmation
- Remove system tray and replace with normal minimize + clean exit flow
- Add force unlock option for stale or locked sessions
- Ensure SQLite vacuum and connection pool clearing before file upload
- Update App.xaml.cs, MainWindow.xaml.cs, Splash.xaml.cs for new flow
- Add localization strings for all sync‑related user prompts (EN/FR)
- Integrate with existing Google Drive service and backup system

Closes: #66
</commit_message>
<xml_diff>
--- a/Source/SKAuto.UI/Localization/Eng_French-Mapping.xlsx
+++ b/Source/SKAuto.UI/Localization/Eng_French-Mapping.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Non Theocratic\SK Auto\Program\SKAutoWorkTracking\Source\SKAuto.UI\Localization\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{358E268E-475B-4C41-A9BB-75778A815C5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B63EE4C5-86AD-4404-A3CF-62715309FE5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ResXResourceManager" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3535" uniqueCount="1508">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3660" uniqueCount="1565">
   <si>
     <t>Project</t>
   </si>
@@ -2137,10 +2137,10 @@
     <t>SK Auto Work Tracking</t>
   </si>
   <si>
-    <t>MainWindow_Footer</t>
-  </si>
-  <si>
-    <t>SK Auto Work Tracking v1.0 – © 2026 Insights®</t>
+    <t>Insights</t>
+  </si>
+  <si>
+    <t>© 2026 Insights®</t>
   </si>
   <si>
     <t>Splash_Title</t>
@@ -2590,13 +2590,13 @@
     <t>Code de vérification :</t>
   </si>
   <si>
-    <t>HelpView_Version</t>
-  </si>
-  <si>
-    <t>Version: 1.0.0 (latest)</t>
-  </si>
-  <si>
-    <t>Version : 1.0.0 (dernière)</t>
+    <t>Version</t>
+  </si>
+  <si>
+    <t>Version: 3.0.0 (Latest)</t>
+  </si>
+  <si>
+    <t>Version : 3.0.0 (dernière)</t>
   </si>
   <si>
     <t>MainWindow_Week</t>
@@ -4465,12 +4465,12 @@
     <t>Mot de passe actuel</t>
   </si>
   <si>
+    <t>ResetPassword</t>
+  </si>
+  <si>
     <t>Reset Password</t>
   </si>
   <si>
-    <t>ResetPassword</t>
-  </si>
-  <si>
     <t>Réinitialiser le mdp</t>
   </si>
   <si>
@@ -4483,7 +4483,17 @@
     <t>Envoyer le code</t>
   </si>
   <si>
-    <t>CodeEmailBody</t>
+    <t>CodeEmailBodyPart1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  &lt;h2&gt;Password Reset Request&lt;/h2&gt;
+                    &lt;p&gt;You requested to reset your password for SKAuto Work Tracking.&lt;/p&gt;
+                    &lt;p&gt;Your verification code is: &lt;strong&gt;</t>
+  </si>
+  <si>
+    <t>&lt;h2&gt;Demande de réinitialisation de mot de passe&lt;/h2&gt;
+&lt;p&gt;Vous avez demandé la réinitialisation de votre mot de passe pour SKAuto Work Tracking.&lt;/p&gt;
+&lt;p&gt;Votre code de vérification est : &lt;strong&gt;</t>
   </si>
   <si>
     <t>CodeEmailTitle</t>
@@ -4495,22 +4505,22 @@
     <t>SKAuto – Code de réinitialisation du mot de passe</t>
   </si>
   <si>
+    <t>CodeSent</t>
+  </si>
+  <si>
     <t>Code Sent</t>
   </si>
   <si>
     <t>Code envoyé</t>
   </si>
   <si>
-    <t>A verification code has been sent to {user.Email}. Please check your inbox.</t>
-  </si>
-  <si>
-    <t>Un code de vérification a été envoyé à {user.Email}. Veuillez consulter votre boîte de réception.</t>
-  </si>
-  <si>
-    <t>CodeSent</t>
-  </si>
-  <si>
-    <t>CodeSentMessageBodySuccess</t>
+    <t>CodeSentMessageBodySuccessPart1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A verification code has been sent to </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Un code de vérification a été envoyé à </t>
   </si>
   <si>
     <t>CodeSentMessageBodyFailed</t>
@@ -4540,27 +4550,186 @@
     <t>Vérifier et réinitialiser</t>
   </si>
   <si>
-    <t xml:space="preserve">
-                    &lt;h2&gt;Password Reset Request&lt;/h2&gt;
-                    &lt;p&gt;You requested to reset your password for SKAuto Work Tracking.&lt;/p&gt;
-                    &lt;p&gt;Your verification code is: &lt;strong&gt;{code}&lt;/strong&gt;&lt;/p&gt;
+    <t>CodeEmailBodyPart2</t>
+  </si>
+  <si>
+    <t>&lt;/strong&gt;&lt;/p&gt;
                     &lt;p&gt;This code will expire in 15 minutes.&lt;/p&gt;
                     &lt;p&gt;If you did not request this, please ignore this email.&lt;/p&gt;</t>
   </si>
   <si>
-    <t xml:space="preserve">
-&lt;h2&gt;Demande de réinitialisation de mot de passe&lt;/h2&gt;
-&lt;p&gt;Vous avez demandé la réinitialisation de votre mot de passe pour SKAuto Work Tracking.&lt;/p&gt;
-&lt;p&gt;Votre code de vérification est : &lt;strong&gt;{code}&lt;/strong&gt;&lt;/p&gt;
+    <t>&lt;/strong&gt;&lt;/p&gt;
 &lt;p&gt;Ce code expirera dans 15 minutes.&lt;/p&gt;
 &lt;p&gt;Si vous n'êtes pas à l'origine de cette demande, veuillez ignorer cet e-mail.&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t>CodeSentMessageBodySuccessPart2</t>
+  </si>
+  <si>
+    <t>Please check your inbox.</t>
+  </si>
+  <si>
+    <t>Veuillez consulter votre boîte de réception.</t>
+  </si>
+  <si>
+    <t>Internet connection is required to verify the database state. Please check your connection and try again.</t>
+  </si>
+  <si>
+    <t>Une connexion Internet est requise pour vérifier l'état de la base de données. Veuillez vérifier votre connexion et réessayer.</t>
+  </si>
+  <si>
+    <t>Sync_ConnectionError</t>
+  </si>
+  <si>
+    <t>Connection Error</t>
+  </si>
+  <si>
+    <t>Erreur de connexion</t>
+  </si>
+  <si>
+    <t>Sync_InternetUnavailable</t>
+  </si>
+  <si>
+    <t>Internet connection is not available. The application cannot start.</t>
+  </si>
+  <si>
+    <t>La connexion Internet n'est pas disponible. L'application ne peut pas démarrer.</t>
+  </si>
+  <si>
+    <t>Sync_LockActive</t>
+  </si>
+  <si>
+    <t>The application is currently in use by {0} on machine {1}. Only one user can use the application at a time.</t>
+  </si>
+  <si>
+    <t>L'application est actuellement utilisée par {0} sur la machine {1}. Un seul utilisateur peut utiliser l'application à la fois.</t>
+  </si>
+  <si>
+    <t>Sync_LockTitle</t>
+  </si>
+  <si>
+    <t>Application in Use</t>
+  </si>
+  <si>
+    <t>Application en cours d'utilisation</t>
+  </si>
+  <si>
+    <t>Sync_StaleLockPrompt</t>
+  </si>
+  <si>
+    <t>A previous session from {0} timed out unexpectedly. This may be due to a crash or network interruption. Do you want to force unlock and continue?</t>
+  </si>
+  <si>
+    <t>Une session précédente de {0} a expiré de manière inattendue. Cela peut être dû à un plantage ou à une interruption réseau. Voulez-vous forcer le déverrouillage et continuer ?</t>
+  </si>
+  <si>
+    <t>Sync_LockFailed</t>
+  </si>
+  <si>
+    <t>Failed to acquire cloud lock. Please check your network connection and try again.</t>
+  </si>
+  <si>
+    <t>Échec de l'acquisition du verrou cloud. Veuillez vérifier votre connexion réseau et réessayer.</t>
+  </si>
+  <si>
+    <t>Sync_ErrorTitle</t>
+  </si>
+  <si>
+    <t>Synchronization Error</t>
+  </si>
+  <si>
+    <t>Erreur de synchronisation</t>
+  </si>
+  <si>
+    <t>Sync_ConflictMessage</t>
+  </si>
+  <si>
+    <t>A version conflict was detected between your local database (v{0}) and the remote database (v{1}).\n\nYour local changes have been backed up to:\n{2}\n\nDo you want to download the remote version (recommended)?</t>
+  </si>
+  <si>
+    <t>Un conflit de version a été détecté entre votre base de données locale (v{0}) et la base de données distante (v{1}).\n\nVos modifications locales ont été sauvegardées dans :\n{2}\n\nVoulez-vous télécharger la version distante (recommandé) ?</t>
+  </si>
+  <si>
+    <t>Sync_ConflictTitle</t>
+  </si>
+  <si>
+    <t>Version Conflict</t>
+  </si>
+  <si>
+    <t>Conflit de version</t>
+  </si>
+  <si>
+    <t>Sync_Error</t>
+  </si>
+  <si>
+    <t>Synchronization failed: {0}</t>
+  </si>
+  <si>
+    <t>La synchronisation a échoué : {0}</t>
+  </si>
+  <si>
+    <t>Sync_ExitError</t>
+  </si>
+  <si>
+    <t>Failed to synchronize database on exit: {0}. Your local changes may not be available on other machines.</t>
+  </si>
+  <si>
+    <t>Échec de la synchronisation de la base de données à la sortie : {0}. Vos modifications locales peuvent ne pas être disponibles sur d'autres machines.</t>
+  </si>
+  <si>
+    <t>Sync_InternetRequired</t>
+  </si>
+  <si>
+    <t>Sync_ForceUnlockQuestion</t>
+  </si>
+  <si>
+    <t>Sync_ForceUnlockFailed</t>
+  </si>
+  <si>
+    <t>Sync_ExitSuccess</t>
+  </si>
+  <si>
+    <t>Sync_SuccessTitle</t>
+  </si>
+  <si>
+    <t>The application appears to be in use by another user or a previous session may have crashed.\n\nDo you want to force unlock and continue? (Use with caution!)</t>
+  </si>
+  <si>
+    <t>Failed to force unlock. Please try again later.</t>
+  </si>
+  <si>
+    <t>Application closed successfully and database synchronized.</t>
+  </si>
+  <si>
+    <t>Success</t>
+  </si>
+  <si>
+    <t>Succès</t>
+  </si>
+  <si>
+    <t>Application fermée avec succès et base de données synchronisée.</t>
+  </si>
+  <si>
+    <t>Échec du déverrouillage forcé. Veuillez réessayer plus tard.</t>
+  </si>
+  <si>
+    <t>L'application semble être utilisée par un autre utilisateur ou une session précédente a peut‑être planté.\n\nVoulez‑vous forcer le déverrouillage et continuer ? (À utiliser avec prudence !)</t>
+  </si>
+  <si>
+    <t>Sync_ExitErrorGeneral</t>
+  </si>
+  <si>
+    <t>The application exited but the database synchronization may have failed. Check the log for details</t>
+  </si>
+  <si>
+    <t>L'application s'est fermée mais la synchronisation de la base de données a peut‑être échoué. Consultez le journal pour plus de détail</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -4568,13 +4737,30 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF0F1115"/>
+      <name val="Inter"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF0F1115"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -4589,13 +4775,20 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyProtection="1">
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1" applyProtection="1">
-      <alignment wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
   </cellXfs>
@@ -4932,14 +5125,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G509"/>
+  <dimension ref="A1:G528"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.28515625" customWidth="1"/>
+    <col min="2" max="2" width="19.85546875" customWidth="1"/>
     <col min="3" max="3" width="44.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="124.7109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="163.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="151.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="175.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
@@ -16328,241 +16521,655 @@
       </c>
     </row>
     <row r="496" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A496" t="s">
-        <v>7</v>
-      </c>
-      <c r="B496" t="s">
-        <v>8</v>
-      </c>
-      <c r="C496" t="s">
+      <c r="A496" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B496" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C496" s="1" t="s">
         <v>1466</v>
+      </c>
+      <c r="D496" t="s">
+        <v>4</v>
       </c>
       <c r="E496" t="s">
         <v>1467</v>
       </c>
+      <c r="F496" t="s">
+        <v>4</v>
+      </c>
       <c r="G496" t="s">
         <v>1468</v>
       </c>
     </row>
     <row r="497" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A497" t="s">
-        <v>7</v>
-      </c>
-      <c r="B497" t="s">
-        <v>8</v>
-      </c>
-      <c r="C497" t="s">
+      <c r="A497" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B497" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C497" s="1" t="s">
         <v>1469</v>
+      </c>
+      <c r="D497" t="s">
+        <v>4</v>
       </c>
       <c r="E497" t="s">
         <v>1470</v>
       </c>
+      <c r="F497" t="s">
+        <v>4</v>
+      </c>
       <c r="G497" t="s">
         <v>1471</v>
       </c>
     </row>
     <row r="498" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A498" t="s">
-        <v>7</v>
-      </c>
-      <c r="B498" t="s">
-        <v>8</v>
-      </c>
-      <c r="C498" t="s">
+      <c r="A498" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B498" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C498" s="1" t="s">
         <v>1472</v>
+      </c>
+      <c r="D498" t="s">
+        <v>4</v>
       </c>
       <c r="E498" t="s">
         <v>1473</v>
       </c>
+      <c r="F498" t="s">
+        <v>4</v>
+      </c>
       <c r="G498" t="s">
         <v>1474</v>
       </c>
     </row>
     <row r="499" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A499" t="s">
-        <v>7</v>
-      </c>
-      <c r="B499" t="s">
-        <v>8</v>
-      </c>
-      <c r="C499" t="s">
+      <c r="A499" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B499" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C499" s="1" t="s">
         <v>1475</v>
+      </c>
+      <c r="D499" t="s">
+        <v>4</v>
       </c>
       <c r="E499" t="s">
         <v>1476</v>
       </c>
+      <c r="F499" t="s">
+        <v>4</v>
+      </c>
       <c r="G499" t="s">
         <v>1477</v>
       </c>
     </row>
     <row r="500" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A500" t="s">
-        <v>7</v>
-      </c>
-      <c r="B500" t="s">
-        <v>8</v>
-      </c>
-      <c r="C500" t="s">
+      <c r="A500" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B500" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C500" s="1" t="s">
         <v>1478</v>
+      </c>
+      <c r="D500" t="s">
+        <v>4</v>
       </c>
       <c r="E500" t="s">
         <v>1479</v>
       </c>
+      <c r="F500" t="s">
+        <v>4</v>
+      </c>
       <c r="G500" t="s">
         <v>1480</v>
       </c>
     </row>
     <row r="501" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A501" t="s">
-        <v>7</v>
-      </c>
-      <c r="B501" t="s">
-        <v>8</v>
-      </c>
-      <c r="C501" t="s">
+      <c r="A501" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B501" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C501" s="1" t="s">
+        <v>1481</v>
+      </c>
+      <c r="D501" t="s">
+        <v>4</v>
+      </c>
+      <c r="E501" t="s">
         <v>1482</v>
       </c>
-      <c r="E501" t="s">
-        <v>1481</v>
+      <c r="F501" t="s">
+        <v>4</v>
       </c>
       <c r="G501" t="s">
         <v>1483</v>
       </c>
     </row>
     <row r="502" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A502" t="s">
-        <v>7</v>
-      </c>
-      <c r="B502" t="s">
-        <v>8</v>
-      </c>
-      <c r="C502" t="s">
+      <c r="A502" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B502" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C502" s="1" t="s">
         <v>1484</v>
+      </c>
+      <c r="D502" t="s">
+        <v>4</v>
       </c>
       <c r="E502" t="s">
         <v>1485</v>
       </c>
+      <c r="F502" t="s">
+        <v>4</v>
+      </c>
       <c r="G502" t="s">
         <v>1486</v>
       </c>
     </row>
-    <row r="503" spans="1:7" ht="90" x14ac:dyDescent="0.25">
-      <c r="A503" t="s">
-        <v>7</v>
-      </c>
-      <c r="B503" t="s">
-        <v>8</v>
-      </c>
-      <c r="C503" t="s">
+    <row r="503" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A503" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B503" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C503" s="1" t="s">
         <v>1487</v>
       </c>
-      <c r="E503" s="2" t="s">
+      <c r="D503" t="s">
+        <v>4</v>
+      </c>
+      <c r="E503" t="s">
+        <v>1488</v>
+      </c>
+      <c r="F503" t="s">
+        <v>4</v>
+      </c>
+      <c r="G503" t="s">
+        <v>1489</v>
+      </c>
+    </row>
+    <row r="504" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A504" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B504" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C504" s="1" t="s">
+        <v>1490</v>
+      </c>
+      <c r="D504" t="s">
+        <v>4</v>
+      </c>
+      <c r="E504" t="s">
+        <v>1491</v>
+      </c>
+      <c r="F504" t="s">
+        <v>4</v>
+      </c>
+      <c r="G504" t="s">
+        <v>1492</v>
+      </c>
+    </row>
+    <row r="505" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A505" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B505" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C505" s="1" t="s">
+        <v>1493</v>
+      </c>
+      <c r="D505" t="s">
+        <v>4</v>
+      </c>
+      <c r="E505" t="s">
+        <v>1494</v>
+      </c>
+      <c r="F505" t="s">
+        <v>4</v>
+      </c>
+      <c r="G505" t="s">
+        <v>1495</v>
+      </c>
+    </row>
+    <row r="506" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A506" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B506" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C506" s="1" t="s">
+        <v>1496</v>
+      </c>
+      <c r="D506" t="s">
+        <v>4</v>
+      </c>
+      <c r="E506" t="s">
+        <v>1497</v>
+      </c>
+      <c r="F506" t="s">
+        <v>4</v>
+      </c>
+      <c r="G506" t="s">
+        <v>1498</v>
+      </c>
+    </row>
+    <row r="507" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A507" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B507" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C507" s="1" t="s">
+        <v>1499</v>
+      </c>
+      <c r="D507" t="s">
+        <v>4</v>
+      </c>
+      <c r="E507" t="s">
+        <v>1500</v>
+      </c>
+      <c r="F507" t="s">
+        <v>4</v>
+      </c>
+      <c r="G507" t="s">
+        <v>1501</v>
+      </c>
+    </row>
+    <row r="508" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A508" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B508" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C508" s="1" t="s">
+        <v>1502</v>
+      </c>
+      <c r="D508" t="s">
+        <v>4</v>
+      </c>
+      <c r="E508" t="s">
+        <v>1503</v>
+      </c>
+      <c r="F508" t="s">
+        <v>4</v>
+      </c>
+      <c r="G508" t="s">
+        <v>1504</v>
+      </c>
+    </row>
+    <row r="509" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A509" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B509" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C509" s="1" t="s">
+        <v>1505</v>
+      </c>
+      <c r="D509" t="s">
+        <v>4</v>
+      </c>
+      <c r="E509" t="s">
         <v>1506</v>
       </c>
-      <c r="G503" s="2" t="s">
+      <c r="F509" t="s">
+        <v>4</v>
+      </c>
+      <c r="G509" t="s">
         <v>1507</v>
       </c>
     </row>
-    <row r="504" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A504" t="s">
-        <v>7</v>
-      </c>
-      <c r="B504" t="s">
-        <v>8</v>
-      </c>
-      <c r="C504" t="s">
-        <v>1488</v>
-      </c>
-      <c r="E504" t="s">
-        <v>1489</v>
-      </c>
-      <c r="G504" t="s">
-        <v>1490</v>
-      </c>
-    </row>
-    <row r="505" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A505" t="s">
-        <v>7</v>
-      </c>
-      <c r="B505" t="s">
-        <v>8</v>
-      </c>
-      <c r="C505" t="s">
-        <v>1495</v>
-      </c>
-      <c r="E505" t="s">
-        <v>1491</v>
-      </c>
-      <c r="G505" t="s">
-        <v>1492</v>
-      </c>
-    </row>
-    <row r="506" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A506" t="s">
-        <v>7</v>
-      </c>
-      <c r="B506" t="s">
-        <v>8</v>
-      </c>
-      <c r="C506" t="s">
-        <v>1496</v>
-      </c>
-      <c r="E506" t="s">
-        <v>1493</v>
-      </c>
-      <c r="G506" t="s">
-        <v>1494</v>
-      </c>
-    </row>
-    <row r="507" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A507" t="s">
-        <v>7</v>
-      </c>
-      <c r="B507" t="s">
-        <v>8</v>
-      </c>
-      <c r="C507" t="s">
-        <v>1497</v>
-      </c>
-      <c r="E507" t="s">
-        <v>1498</v>
-      </c>
-      <c r="G507" t="s">
-        <v>1499</v>
-      </c>
-    </row>
-    <row r="508" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A508" t="s">
-        <v>7</v>
-      </c>
-      <c r="B508" t="s">
-        <v>8</v>
-      </c>
-      <c r="C508" t="s">
-        <v>1500</v>
-      </c>
-      <c r="E508" t="s">
-        <v>1501</v>
-      </c>
-      <c r="G508" t="s">
-        <v>1502</v>
-      </c>
-    </row>
-    <row r="509" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A509" t="s">
-        <v>7</v>
-      </c>
-      <c r="B509" t="s">
-        <v>8</v>
-      </c>
-      <c r="C509" t="s">
-        <v>1503</v>
-      </c>
-      <c r="E509" t="s">
-        <v>1504</v>
-      </c>
-      <c r="G509" t="s">
-        <v>1505</v>
+    <row r="510" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A510" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B510" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C510" s="1" t="s">
+        <v>1508</v>
+      </c>
+      <c r="D510" t="s">
+        <v>4</v>
+      </c>
+      <c r="E510" t="s">
+        <v>1509</v>
+      </c>
+      <c r="F510" t="s">
+        <v>4</v>
+      </c>
+      <c r="G510" t="s">
+        <v>1510</v>
+      </c>
+    </row>
+    <row r="511" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A511" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B511" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C511" s="1" t="s">
+        <v>1511</v>
+      </c>
+      <c r="D511" t="s">
+        <v>4</v>
+      </c>
+      <c r="E511" t="s">
+        <v>1512</v>
+      </c>
+      <c r="F511" t="s">
+        <v>4</v>
+      </c>
+      <c r="G511" t="s">
+        <v>1513</v>
+      </c>
+    </row>
+    <row r="512" spans="1:7" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="A512" t="s">
+        <v>7</v>
+      </c>
+      <c r="B512" t="s">
+        <v>8</v>
+      </c>
+      <c r="C512" s="2" t="s">
+        <v>1549</v>
+      </c>
+      <c r="E512" s="3" t="s">
+        <v>1514</v>
+      </c>
+      <c r="G512" s="3" t="s">
+        <v>1515</v>
+      </c>
+    </row>
+    <row r="513" spans="1:7" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="A513" t="s">
+        <v>7</v>
+      </c>
+      <c r="B513" t="s">
+        <v>8</v>
+      </c>
+      <c r="C513" s="2" t="s">
+        <v>1516</v>
+      </c>
+      <c r="E513" s="3" t="s">
+        <v>1517</v>
+      </c>
+      <c r="G513" s="3" t="s">
+        <v>1518</v>
+      </c>
+    </row>
+    <row r="514" spans="1:7" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="A514" t="s">
+        <v>7</v>
+      </c>
+      <c r="B514" t="s">
+        <v>8</v>
+      </c>
+      <c r="C514" s="2" t="s">
+        <v>1519</v>
+      </c>
+      <c r="E514" s="3" t="s">
+        <v>1520</v>
+      </c>
+      <c r="G514" s="3" t="s">
+        <v>1521</v>
+      </c>
+    </row>
+    <row r="515" spans="1:7" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="A515" t="s">
+        <v>7</v>
+      </c>
+      <c r="B515" t="s">
+        <v>8</v>
+      </c>
+      <c r="C515" s="2" t="s">
+        <v>1522</v>
+      </c>
+      <c r="E515" s="3" t="s">
+        <v>1523</v>
+      </c>
+      <c r="G515" s="3" t="s">
+        <v>1524</v>
+      </c>
+    </row>
+    <row r="516" spans="1:7" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="A516" t="s">
+        <v>7</v>
+      </c>
+      <c r="B516" t="s">
+        <v>8</v>
+      </c>
+      <c r="C516" s="2" t="s">
+        <v>1525</v>
+      </c>
+      <c r="E516" s="3" t="s">
+        <v>1526</v>
+      </c>
+      <c r="G516" s="3" t="s">
+        <v>1527</v>
+      </c>
+    </row>
+    <row r="517" spans="1:7" ht="37.5" x14ac:dyDescent="0.25">
+      <c r="A517" t="s">
+        <v>7</v>
+      </c>
+      <c r="B517" t="s">
+        <v>8</v>
+      </c>
+      <c r="C517" s="2" t="s">
+        <v>1528</v>
+      </c>
+      <c r="E517" s="3" t="s">
+        <v>1529</v>
+      </c>
+      <c r="G517" s="3" t="s">
+        <v>1530</v>
+      </c>
+    </row>
+    <row r="518" spans="1:7" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="A518" t="s">
+        <v>7</v>
+      </c>
+      <c r="B518" t="s">
+        <v>8</v>
+      </c>
+      <c r="C518" s="2" t="s">
+        <v>1531</v>
+      </c>
+      <c r="E518" s="3" t="s">
+        <v>1532</v>
+      </c>
+      <c r="G518" s="3" t="s">
+        <v>1533</v>
+      </c>
+    </row>
+    <row r="519" spans="1:7" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="A519" t="s">
+        <v>7</v>
+      </c>
+      <c r="B519" t="s">
+        <v>8</v>
+      </c>
+      <c r="C519" s="2" t="s">
+        <v>1534</v>
+      </c>
+      <c r="E519" s="3" t="s">
+        <v>1535</v>
+      </c>
+      <c r="G519" s="3" t="s">
+        <v>1536</v>
+      </c>
+    </row>
+    <row r="520" spans="1:7" ht="37.5" x14ac:dyDescent="0.25">
+      <c r="A520" t="s">
+        <v>7</v>
+      </c>
+      <c r="B520" t="s">
+        <v>8</v>
+      </c>
+      <c r="C520" s="2" t="s">
+        <v>1537</v>
+      </c>
+      <c r="E520" s="3" t="s">
+        <v>1538</v>
+      </c>
+      <c r="G520" s="3" t="s">
+        <v>1539</v>
+      </c>
+    </row>
+    <row r="521" spans="1:7" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="A521" t="s">
+        <v>7</v>
+      </c>
+      <c r="B521" t="s">
+        <v>8</v>
+      </c>
+      <c r="C521" s="2" t="s">
+        <v>1540</v>
+      </c>
+      <c r="E521" s="3" t="s">
+        <v>1541</v>
+      </c>
+      <c r="G521" s="3" t="s">
+        <v>1542</v>
+      </c>
+    </row>
+    <row r="522" spans="1:7" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="A522" t="s">
+        <v>7</v>
+      </c>
+      <c r="B522" t="s">
+        <v>8</v>
+      </c>
+      <c r="C522" s="2" t="s">
+        <v>1543</v>
+      </c>
+      <c r="E522" s="3" t="s">
+        <v>1544</v>
+      </c>
+      <c r="G522" s="3" t="s">
+        <v>1545</v>
+      </c>
+    </row>
+    <row r="523" spans="1:7" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="A523" t="s">
+        <v>7</v>
+      </c>
+      <c r="B523" t="s">
+        <v>8</v>
+      </c>
+      <c r="C523" s="2" t="s">
+        <v>1546</v>
+      </c>
+      <c r="E523" s="3" t="s">
+        <v>1547</v>
+      </c>
+      <c r="G523" s="3" t="s">
+        <v>1548</v>
+      </c>
+    </row>
+    <row r="524" spans="1:7" ht="37.5" x14ac:dyDescent="0.25">
+      <c r="A524" t="s">
+        <v>7</v>
+      </c>
+      <c r="B524" t="s">
+        <v>8</v>
+      </c>
+      <c r="C524" s="2" t="s">
+        <v>1550</v>
+      </c>
+      <c r="E524" s="3" t="s">
+        <v>1554</v>
+      </c>
+      <c r="G524" s="3" t="s">
+        <v>1561</v>
+      </c>
+    </row>
+    <row r="525" spans="1:7" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="A525" t="s">
+        <v>7</v>
+      </c>
+      <c r="B525" t="s">
+        <v>8</v>
+      </c>
+      <c r="C525" s="2" t="s">
+        <v>1551</v>
+      </c>
+      <c r="E525" s="3" t="s">
+        <v>1555</v>
+      </c>
+      <c r="G525" s="3" t="s">
+        <v>1560</v>
+      </c>
+    </row>
+    <row r="526" spans="1:7" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="A526" t="s">
+        <v>7</v>
+      </c>
+      <c r="B526" t="s">
+        <v>8</v>
+      </c>
+      <c r="C526" s="2" t="s">
+        <v>1552</v>
+      </c>
+      <c r="E526" s="3" t="s">
+        <v>1556</v>
+      </c>
+      <c r="G526" s="3" t="s">
+        <v>1559</v>
+      </c>
+    </row>
+    <row r="527" spans="1:7" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="A527" t="s">
+        <v>7</v>
+      </c>
+      <c r="B527" t="s">
+        <v>8</v>
+      </c>
+      <c r="C527" s="2" t="s">
+        <v>1553</v>
+      </c>
+      <c r="E527" s="3" t="s">
+        <v>1557</v>
+      </c>
+      <c r="G527" s="3" t="s">
+        <v>1558</v>
+      </c>
+    </row>
+    <row r="528" spans="1:7" ht="18.75" x14ac:dyDescent="0.4">
+      <c r="C528" s="2" t="s">
+        <v>1562</v>
+      </c>
+      <c r="D528" s="3"/>
+      <c r="E528" t="s">
+        <v>1563</v>
+      </c>
+      <c r="G528" s="4" t="s">
+        <v>1564</v>
       </c>
     </row>
   </sheetData>

</xml_diff>